<commit_message>
feat(t04): thin FR-003 flower type, colour, ribbon options
Accept catalog-backed flower_type and reference colour/ribbon on the selection path, promote FR-003 to MVP thin scope, and keep gift-card/free-form composition rejected. Closes #22.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/archive/Quantic_Project_Consolidated_Coherence_Validated.xlsx
+++ b/archive/Quantic_Project_Consolidated_Coherence_Validated.xlsx
@@ -1315,1583 +1315,1583 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="14.875" customWidth="1"/>
-    <x:col min="2" max="2" width="55.875" customWidth="1"/>
-    <x:col min="3" max="3" width="12.875" customWidth="1"/>
-    <x:col min="4" max="4" width="45.875" customWidth="1"/>
-    <x:col min="5" max="5" width="90.875" customWidth="1"/>
-    <x:col min="6" max="6" width="18.875" customWidth="1"/>
-    <x:col min="7" max="7" width="110.875" customWidth="1"/>
-    <x:col min="8" max="9" width="18.875" customWidth="1"/>
-    <x:col min="10" max="10" width="110.875" customWidth="1"/>
-    <x:col min="11" max="11" width="25.875" customWidth="1"/>
-    <x:col min="12" max="12" width="14.875" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="15.75">
-      <x:c r="A1" s="7" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B1" s="7" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C1" s="7" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="D1" s="7" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="E1" s="7" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="F1" s="7" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="G1" s="7" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="H1" s="7" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="I1" s="7" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="J1" s="7" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="K1" s="7" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="L1" s="7" t="s">
-        <x:v>58</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="15.75">
-      <x:c r="A2" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B2" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C2" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D2" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E2" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F2" s="12" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G2" s="12" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="H2" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I2" s="12" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="J2" s="12" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="K2" s="12" t="str">
-        <x:v>Discovery and Intent</x:v>
-      </x:c>
-      <x:c r="L2" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="15.75">
-      <x:c r="A3" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D3" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E3" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="G3" s="12" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="H3" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I3" s="12" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="J3" s="12" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="K3" s="12" t="str">
-        <x:v>Discovery and Intent</x:v>
-      </x:c>
-      <x:c r="L3" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15.75">
-      <x:c r="A4" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D4" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F4" s="12" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="G4" s="12" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="H4" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I4" s="12" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="J4" s="12" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="K4" s="12" t="str">
-        <x:v>Customization</x:v>
-      </x:c>
-      <x:c r="L4" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15.75">
-      <x:c r="A5" s="12" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B5" s="12" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C5" s="12" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D5" s="12" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E5" s="12" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F5" s="12" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="G5" s="12" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="H5" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I5" s="12" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="J5" s="12" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="K5" s="12" t="str">
-        <x:v>Discovery and Intent</x:v>
-      </x:c>
-      <x:c r="L5" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15.75">
-      <x:c r="A6" s="12" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B6" s="12" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C6" s="12" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D6" s="12" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E6" s="12" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F6" s="12" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="G6" s="12" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="H6" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I6" s="12" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J6" s="12" t="s">
-        <x:v>81</x:v>
-      </x:c>
-      <x:c r="K6" s="12" t="str">
-        <x:v>Discovery and Intent</x:v>
-      </x:c>
-      <x:c r="L6" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15.75">
-      <x:c r="A7" s="12" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B7" s="12" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C7" s="12" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D7" s="12" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E7" s="12" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F7" s="12" t="s">
-        <x:v>82</x:v>
-      </x:c>
-      <x:c r="G7" s="12" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="H7" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I7" s="12" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="J7" s="12" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="K7" s="12" t="str">
-        <x:v>Support Automation</x:v>
-      </x:c>
-      <x:c r="L7" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15.75">
-      <x:c r="A8" s="12" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B8" s="12" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C8" s="12" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D8" s="12" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E8" s="12" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F8" s="12" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="G8" s="12" t="s">
-        <x:v>87</x:v>
-      </x:c>
-      <x:c r="H8" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I8" s="12" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="J8" s="12" t="s">
-        <x:v>89</x:v>
-      </x:c>
-      <x:c r="K8" s="12" t="str">
-        <x:v>Recommendations</x:v>
-      </x:c>
-      <x:c r="L8" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15.75">
-      <x:c r="A9" s="12" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B9" s="12" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C9" s="12" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D9" s="12" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E9" s="12" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F9" s="12" t="s">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="G9" s="12" t="s">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="H9" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I9" s="12" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="J9" s="12" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="K9" s="12" t="str">
-        <x:v>Recommendations</x:v>
-      </x:c>
-      <x:c r="L9" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15.75">
-      <x:c r="A10" s="12" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B10" s="12" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C10" s="12" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D10" s="12" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E10" s="12" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F10" s="12" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="G10" s="12" t="s">
-        <x:v>95</x:v>
-      </x:c>
-      <x:c r="H10" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I10" s="12" t="s">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="J10" s="12" t="s">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="K10" s="12" t="str">
-        <x:v>Support Automation</x:v>
-      </x:c>
-      <x:c r="L10" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="15.75">
-      <x:c r="A11" s="12" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B11" s="12" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C11" s="12" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D11" s="12" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E11" s="12" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F11" s="12" t="s">
-        <x:v>98</x:v>
-      </x:c>
-      <x:c r="G11" s="12" t="s">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="H11" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I11" s="12" t="s">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="J11" s="12" t="s">
-        <x:v>101</x:v>
-      </x:c>
-      <x:c r="K11" s="12" t="str">
-        <x:v>Support Automation</x:v>
-      </x:c>
-      <x:c r="L11" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15.75">
-      <x:c r="A12" s="12" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B12" s="12" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C12" s="12" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D12" s="12" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="E12" s="12" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F12" s="12" t="s">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="G12" s="12" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="H12" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I12" s="12" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="J12" s="12" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="K12" s="12" t="str">
-        <x:v>Inventory</x:v>
-      </x:c>
-      <x:c r="L12" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="15.75">
-      <x:c r="A13" s="12" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B13" s="12" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C13" s="12" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D13" s="12" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="E13" s="12" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F13" s="12" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="G13" s="12" t="s">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="H13" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I13" s="12" t="s">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="J13" s="12" t="s">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="K13" s="12" t="str">
-        <x:v>Inventory</x:v>
-      </x:c>
-      <x:c r="L13" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="15.75">
-      <x:c r="A14" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B14" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C14" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D14" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E14" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F14" s="12" t="s">
-        <x:v>110</x:v>
-      </x:c>
-      <x:c r="G14" s="12" t="s">
-        <x:v>111</x:v>
-      </x:c>
-      <x:c r="H14" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I14" s="12" t="s">
-        <x:v>112</x:v>
-      </x:c>
-      <x:c r="J14" s="12" t="s">
-        <x:v>113</x:v>
-      </x:c>
-      <x:c r="K14" s="12" t="str">
-        <x:v>Ordering and Delivery</x:v>
-      </x:c>
-      <x:c r="L14" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="15.75">
-      <x:c r="A15" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B15" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C15" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D15" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E15" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F15" s="12" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="G15" s="12" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="H15" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I15" s="12" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="J15" s="12" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="K15" s="12" t="str">
-        <x:v>Ordering and Delivery</x:v>
-      </x:c>
-      <x:c r="L15" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="15.75">
-      <x:c r="A16" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B16" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C16" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D16" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E16" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F16" s="12" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="G16" s="12" t="s">
-        <x:v>119</x:v>
-      </x:c>
-      <x:c r="H16" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I16" s="12" t="s">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="J16" s="12" t="s">
-        <x:v>121</x:v>
-      </x:c>
-      <x:c r="K16" s="12" t="str">
-        <x:v>Ordering and Delivery</x:v>
-      </x:c>
-      <x:c r="L16" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="15.75">
-      <x:c r="A17" s="12" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B17" s="12" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C17" s="12" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D17" s="12" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="E17" s="12" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F17" s="12" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="G17" s="12" t="s">
-        <x:v>123</x:v>
-      </x:c>
-      <x:c r="H17" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I17" s="12" t="s">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="J17" s="12" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="K17" s="12" t="str">
-        <x:v>Engagement and CRM</x:v>
-      </x:c>
-      <x:c r="L17" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15.75">
-      <x:c r="A18" s="12" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B18" s="12" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C18" s="12" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D18" s="12" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="E18" s="12" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F18" s="12" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="G18" s="12" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="H18" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I18" s="12" t="s">
-        <x:v>128</x:v>
-      </x:c>
-      <x:c r="J18" s="12" t="s">
-        <x:v>129</x:v>
-      </x:c>
-      <x:c r="K18" s="12" t="str">
-        <x:v>Engagement and CRM</x:v>
-      </x:c>
-      <x:c r="L18" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="15.75">
-      <x:c r="A19" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B19" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C19" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D19" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E19" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F19" s="12" t="s">
-        <x:v>130</x:v>
-      </x:c>
-      <x:c r="G19" s="12" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="H19" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I19" s="12" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="J19" s="12" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="K19" s="12" t="str">
-        <x:v>Usability</x:v>
-      </x:c>
-      <x:c r="L19" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="15.75">
-      <x:c r="A20" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B20" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C20" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D20" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E20" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F20" s="12" t="s">
-        <x:v>135</x:v>
-      </x:c>
-      <x:c r="G20" s="12" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="H20" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I20" s="12" t="s">
-        <x:v>137</x:v>
-      </x:c>
-      <x:c r="J20" s="12" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="K20" s="12" t="str">
-        <x:v>Compatibility</x:v>
-      </x:c>
-      <x:c r="L20" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="15.75">
-      <x:c r="A21" s="12" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B21" s="12" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C21" s="12" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D21" s="12" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E21" s="12" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F21" s="12" t="s">
-        <x:v>139</x:v>
-      </x:c>
-      <x:c r="G21" s="12" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="H21" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I21" s="12" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="J21" s="12" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="K21" s="12" t="str">
-        <x:v>Availability</x:v>
-      </x:c>
-      <x:c r="L21" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="15.75">
-      <x:c r="A22" s="12" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B22" s="12" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C22" s="12" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D22" s="12" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E22" s="12" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F22" s="12" t="s">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="G22" s="12" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="H22" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I22" s="12" t="s">
-        <x:v>145</x:v>
-      </x:c>
-      <x:c r="J22" s="12" t="s">
-        <x:v>146</x:v>
-      </x:c>
-      <x:c r="K22" s="12" t="str">
-        <x:v>Performance</x:v>
-      </x:c>
-      <x:c r="L22" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="15.75">
-      <x:c r="A23" s="12" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B23" s="12" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C23" s="12" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D23" s="12" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E23" s="12" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F23" s="12" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="G23" s="12" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="H23" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I23" s="12" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="J23" s="12" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="K23" s="12" t="str">
-        <x:v>Transparency</x:v>
-      </x:c>
-      <x:c r="L23" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="15.75">
-      <x:c r="A24" s="12" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B24" s="12" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C24" s="12" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D24" s="12" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E24" s="12" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F24" s="12" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="G24" s="12" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="H24" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I24" s="12" t="s">
-        <x:v>153</x:v>
-      </x:c>
-      <x:c r="J24" s="12" t="s">
-        <x:v>154</x:v>
-      </x:c>
-      <x:c r="K24" s="12" t="str">
-        <x:v>Accuracy</x:v>
-      </x:c>
-      <x:c r="L24" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="15.75">
-      <x:c r="A25" s="12" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B25" s="12" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="C25" s="12" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D25" s="12" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E25" s="12" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F25" s="12" t="s">
-        <x:v>155</x:v>
-      </x:c>
-      <x:c r="G25" s="12" t="s">
-        <x:v>156</x:v>
-      </x:c>
-      <x:c r="H25" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I25" s="12" t="s">
-        <x:v>157</x:v>
-      </x:c>
-      <x:c r="J25" s="12" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="K25" s="12" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="L25" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="15.75">
-      <x:c r="A26" s="12" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B26" s="12" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="C26" s="12" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="D26" s="12" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="E26" s="12" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="F26" s="12" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="G26" s="12" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="H26" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I26" s="12" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="J26" s="12" t="s">
-        <x:v>162</x:v>
-      </x:c>
-      <x:c r="K26" s="12" t="str">
-        <x:v>Reliability</x:v>
-      </x:c>
-      <x:c r="L26" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="15.75">
-      <x:c r="A27" s="12" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B27" s="12" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C27" s="12" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D27" s="12" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="E27" s="12" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F27" s="12" t="s">
-        <x:v>163</x:v>
-      </x:c>
-      <x:c r="G27" s="12" t="s">
-        <x:v>164</x:v>
-      </x:c>
-      <x:c r="H27" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I27" s="12" t="s">
-        <x:v>165</x:v>
-      </x:c>
-      <x:c r="J27" s="12" t="s">
-        <x:v>166</x:v>
-      </x:c>
-      <x:c r="K27" s="12" t="str">
-        <x:v>Data Integrity</x:v>
-      </x:c>
-      <x:c r="L27" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="15.75">
-      <x:c r="A28" s="12" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="B28" s="12" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="C28" s="12" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D28" s="12" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="E28" s="12" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="F28" s="12" t="s">
-        <x:v>167</x:v>
-      </x:c>
-      <x:c r="G28" s="12" t="s">
-        <x:v>168</x:v>
-      </x:c>
-      <x:c r="H28" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I28" s="12" t="s">
-        <x:v>169</x:v>
-      </x:c>
-      <x:c r="J28" s="12" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="K28" s="12" t="str">
-        <x:v>Reliability</x:v>
-      </x:c>
-      <x:c r="L28" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="15.75">
-      <x:c r="A29" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B29" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C29" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D29" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E29" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F29" s="12" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="G29" s="12" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="H29" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I29" s="12" t="s">
-        <x:v>173</x:v>
-      </x:c>
-      <x:c r="J29" s="12" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="K29" s="12" t="str">
-        <x:v>Performance</x:v>
-      </x:c>
-      <x:c r="L29" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="15.75">
-      <x:c r="A30" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B30" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C30" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D30" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E30" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F30" s="12" t="s">
-        <x:v>175</x:v>
-      </x:c>
-      <x:c r="G30" s="12" t="s">
-        <x:v>176</x:v>
-      </x:c>
-      <x:c r="H30" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I30" s="12" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="J30" s="12" t="s">
-        <x:v>178</x:v>
-      </x:c>
-      <x:c r="K30" s="12" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="L30" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15.75">
-      <x:c r="A31" s="12" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B31" s="12" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C31" s="12" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D31" s="12" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="E31" s="12" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F31" s="12" t="s">
-        <x:v>179</x:v>
-      </x:c>
-      <x:c r="G31" s="12" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="H31" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I31" s="12" t="s">
-        <x:v>181</x:v>
-      </x:c>
-      <x:c r="J31" s="12" t="s">
-        <x:v>182</x:v>
-      </x:c>
-      <x:c r="K31" s="12" t="str">
-        <x:v>Security</x:v>
-      </x:c>
-      <x:c r="L31" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15.75">
-      <x:c r="A32" s="12" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="B32" s="12" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="C32" s="12" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="D32" s="12" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="E32" s="12" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F32" s="12" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="G32" s="12" t="s">
-        <x:v>184</x:v>
-      </x:c>
-      <x:c r="H32" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I32" s="12" t="s">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="J32" s="12" t="s">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="K32" s="12" t="str">
-        <x:v>Scalability</x:v>
-      </x:c>
-      <x:c r="L32" s="12" t="s">
-        <x:v>73</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15.75">
-      <x:c r="A33" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B33" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C33" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D33" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E33" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F33" s="12" t="s">
-        <x:v>187</x:v>
-      </x:c>
-      <x:c r="G33" s="12" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="H33" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I33" s="12" t="s">
-        <x:v>189</x:v>
-      </x:c>
-      <x:c r="J33" s="12" t="s">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="K33" s="12" t="str">
-        <x:v>Ordering and Delivery</x:v>
-      </x:c>
-      <x:c r="L33" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="15.75">
-      <x:c r="A34" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B34" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C34" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D34" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E34" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F34" s="12" t="s">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="G34" s="12" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="H34" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I34" s="12" t="s">
-        <x:v>193</x:v>
-      </x:c>
-      <x:c r="J34" s="12" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="K34" s="12" t="str">
-        <x:v>Ordering and Delivery</x:v>
-      </x:c>
-      <x:c r="L34" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="15.75">
-      <x:c r="A35" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B35" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C35" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D35" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E35" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F35" s="12" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="G35" s="12" t="s">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="H35" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I35" s="12" t="s">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="J35" s="12" t="s">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="K35" s="12" t="str">
-        <x:v>Workspace Behavior</x:v>
-      </x:c>
-      <x:c r="L35" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="15.75">
-      <x:c r="A36" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B36" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C36" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D36" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E36" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F36" s="12" t="s">
-        <x:v>199</x:v>
-      </x:c>
-      <x:c r="G36" s="12" t="s">
-        <x:v>200</x:v>
-      </x:c>
-      <x:c r="H36" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I36" s="12" t="s">
-        <x:v>201</x:v>
-      </x:c>
-      <x:c r="J36" s="12" t="s">
-        <x:v>202</x:v>
-      </x:c>
-      <x:c r="K36" s="12" t="str">
-        <x:v>Workspace Behavior</x:v>
-      </x:c>
-      <x:c r="L36" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="15.75">
-      <x:c r="A37" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B37" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C37" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D37" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E37" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F37" s="12" t="s">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="G37" s="12" t="s">
-        <x:v>204</x:v>
-      </x:c>
-      <x:c r="H37" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I37" s="12" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="J37" s="12" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="K37" s="12" t="str">
-        <x:v>Workspace Behavior</x:v>
-      </x:c>
-      <x:c r="L37" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="15.75">
-      <x:c r="A38" s="12" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="B38" s="12" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C38" s="12" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D38" s="12" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="E38" s="12" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="F38" s="12" t="s">
-        <x:v>207</x:v>
-      </x:c>
-      <x:c r="G38" s="12" t="s">
-        <x:v>208</x:v>
-      </x:c>
-      <x:c r="H38" s="12" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="I38" s="12" t="s">
-        <x:v>209</x:v>
-      </x:c>
-      <x:c r="J38" s="12" t="s">
-        <x:v>210</x:v>
-      </x:c>
-      <x:c r="K38" s="12" t="str">
-        <x:v>Order Tracking</x:v>
-      </x:c>
-      <x:c r="L38" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="15.75">
-      <x:c r="A39" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B39" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C39" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D39" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E39" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F39" s="12" t="s">
-        <x:v>211</x:v>
-      </x:c>
-      <x:c r="G39" s="12" t="s">
-        <x:v>212</x:v>
-      </x:c>
-      <x:c r="H39" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I39" s="12" t="s">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="J39" s="12" t="s">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="K39" s="12" t="str">
-        <x:v>Maintainability / Governance</x:v>
-      </x:c>
-      <x:c r="L39" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="15.75">
-      <x:c r="A40" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B40" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C40" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D40" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E40" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F40" s="12" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="G40" s="12" t="s">
-        <x:v>216</x:v>
-      </x:c>
-      <x:c r="H40" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I40" s="12" t="s">
-        <x:v>217</x:v>
-      </x:c>
-      <x:c r="J40" s="12" t="s">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="K40" s="12" t="str">
-        <x:v>Observability / Auditability</x:v>
-      </x:c>
-      <x:c r="L40" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="15.75">
-      <x:c r="A41" s="12" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B41" s="12" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C41" s="12" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="D41" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="E41" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F41" s="12" t="s">
-        <x:v>219</x:v>
-      </x:c>
-      <x:c r="G41" s="12" t="s">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="H41" s="12" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="I41" s="12" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="J41" s="12" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="K41" s="12" t="str">
-        <x:v>Privacy / Security</x:v>
-      </x:c>
-      <x:c r="L41" s="12" t="s">
-        <x:v>64</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.875" customWidth="1"/>
+    <col min="2" max="2" width="55.875" customWidth="1"/>
+    <col min="3" max="3" width="12.875" customWidth="1"/>
+    <col min="4" max="4" width="45.875" customWidth="1"/>
+    <col min="5" max="5" width="90.875" customWidth="1"/>
+    <col min="6" max="6" width="18.875" customWidth="1"/>
+    <col min="7" max="7" width="110.875" customWidth="1"/>
+    <col min="8" max="9" width="18.875" customWidth="1"/>
+    <col min="10" max="10" width="110.875" customWidth="1"/>
+    <col min="11" max="11" width="25.875" customWidth="1"/>
+    <col min="12" max="12" width="14.875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.75">
+      <c r="A1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75">
+      <c r="A2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K2" s="12" t="str">
+        <v>Discovery and Intent</v>
+      </c>
+      <c r="L2" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75">
+      <c r="A3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="K3" s="12" t="str">
+        <v>Discovery and Intent</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75">
+      <c r="A4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="K4" s="12" t="str">
+        <v>Customization</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75">
+      <c r="A5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="J5" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="K5" s="12" t="str">
+        <v>Discovery and Intent</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75">
+      <c r="A6" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="K6" s="12" t="str">
+        <v>Discovery and Intent</v>
+      </c>
+      <c r="L6" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75">
+      <c r="A7" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="K7" s="12" t="str">
+        <v>Support Automation</v>
+      </c>
+      <c r="L7" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75">
+      <c r="A8" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="K8" s="12" t="str">
+        <v>Recommendations</v>
+      </c>
+      <c r="L8" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75">
+      <c r="A9" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="K9" s="12" t="str">
+        <v>Recommendations</v>
+      </c>
+      <c r="L9" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75">
+      <c r="A10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="K10" s="12" t="str">
+        <v>Support Automation</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75">
+      <c r="A11" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>98</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I11" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="K11" s="12" t="str">
+        <v>Support Automation</v>
+      </c>
+      <c r="L11" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75">
+      <c r="A12" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="K12" s="12" t="str">
+        <v>Inventory</v>
+      </c>
+      <c r="L12" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75">
+      <c r="A13" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I13" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="J13" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="K13" s="12" t="str">
+        <v>Inventory</v>
+      </c>
+      <c r="L13" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75">
+      <c r="A14" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="K14" s="12" t="str">
+        <v>Ordering and Delivery</v>
+      </c>
+      <c r="L14" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" ht="15.75">
+      <c r="A15" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G15" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="J15" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="K15" s="12" t="str">
+        <v>Ordering and Delivery</v>
+      </c>
+      <c r="L15" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" ht="15.75">
+      <c r="A16" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I16" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="K16" s="12" t="str">
+        <v>Ordering and Delivery</v>
+      </c>
+      <c r="L16" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" ht="15.75">
+      <c r="A17" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="G17" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="K17" s="12" t="str">
+        <v>Engagement and CRM</v>
+      </c>
+      <c r="L17" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75">
+      <c r="A18" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="G18" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="K18" s="12" t="str">
+        <v>Engagement and CRM</v>
+      </c>
+      <c r="L18" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" ht="15.75">
+      <c r="A19" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I19" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="J19" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="K19" s="12" t="str">
+        <v>Usability</v>
+      </c>
+      <c r="L19" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75">
+      <c r="A20" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I20" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>138</v>
+      </c>
+      <c r="K20" s="12" t="str">
+        <v>Compatibility</v>
+      </c>
+      <c r="L20" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75">
+      <c r="A21" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="H21" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I21" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="J21" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="K21" s="12" t="str">
+        <v>Availability</v>
+      </c>
+      <c r="L21" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75">
+      <c r="A22" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I22" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="K22" s="12" t="str">
+        <v>Performance</v>
+      </c>
+      <c r="L22" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75">
+      <c r="A23" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="H23" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I23" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="J23" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="K23" s="12" t="str">
+        <v>Transparency</v>
+      </c>
+      <c r="L23" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75">
+      <c r="A24" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I24" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="K24" s="12" t="str">
+        <v>Accuracy</v>
+      </c>
+      <c r="L24" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75">
+      <c r="A25" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I25" s="12" t="s">
+        <v>157</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="K25" s="12" t="str">
+        <v>Security</v>
+      </c>
+      <c r="L25" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75">
+      <c r="A26" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>160</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I26" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="K26" s="12" t="str">
+        <v>Reliability</v>
+      </c>
+      <c r="L26" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75">
+      <c r="A27" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="H27" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I27" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="J27" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="K27" s="12" t="str">
+        <v>Data Integrity</v>
+      </c>
+      <c r="L27" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75">
+      <c r="A28" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I28" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="K28" s="12" t="str">
+        <v>Reliability</v>
+      </c>
+      <c r="L28" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75">
+      <c r="A29" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F29" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I29" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="K29" s="12" t="str">
+        <v>Performance</v>
+      </c>
+      <c r="L29" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75">
+      <c r="A30" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>176</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I30" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="K30" s="12" t="str">
+        <v>Security</v>
+      </c>
+      <c r="L30" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75">
+      <c r="A31" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F31" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="H31" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I31" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="J31" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="K31" s="12" t="str">
+        <v>Security</v>
+      </c>
+      <c r="L31" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75">
+      <c r="A32" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="G32" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="H32" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I32" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="K32" s="12" t="str">
+        <v>Scalability</v>
+      </c>
+      <c r="L32" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75">
+      <c r="A33" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="K33" s="12" t="str">
+        <v>Ordering and Delivery</v>
+      </c>
+      <c r="L33" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75">
+      <c r="A34" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="G34" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I34" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="J34" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="K34" s="12" t="str">
+        <v>Ordering and Delivery</v>
+      </c>
+      <c r="L34" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75">
+      <c r="A35" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E35" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="J35" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="K35" s="12" t="str">
+        <v>Workspace Behavior</v>
+      </c>
+      <c r="L35" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75">
+      <c r="A36" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="J36" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="K36" s="12" t="str">
+        <v>Workspace Behavior</v>
+      </c>
+      <c r="L36" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75">
+      <c r="A37" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I37" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="J37" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="K37" s="12" t="str">
+        <v>Workspace Behavior</v>
+      </c>
+      <c r="L37" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75">
+      <c r="A38" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="B38" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D38" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E38" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="I38" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="J38" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="K38" s="12" t="str">
+        <v>Order Tracking</v>
+      </c>
+      <c r="L38" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75">
+      <c r="A39" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F39" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I39" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="J39" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="K39" s="12" t="str">
+        <v>Maintainability / Governance</v>
+      </c>
+      <c r="L39" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75">
+      <c r="A40" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B40" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="G40" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="H40" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I40" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="J40" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="K40" s="12" t="str">
+        <v>Observability / Auditability</v>
+      </c>
+      <c r="L40" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75">
+      <c r="A41" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B41" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F41" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="G41" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="H41" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I41" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="J41" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="K41" s="12" t="str">
+        <v>Privacy / Security</v>
+      </c>
+      <c r="L41" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>